<commit_message>
feat: update week 6 lab data and implement script to automate laboratory content synchronization
</commit_message>
<xml_diff>
--- a/public/data/week-6a_wayground_import.xlsx
+++ b/public/data/week-6a_wayground_import.xlsx
@@ -984,123 +984,403 @@
       <c r="J12" s="10" t="n"/>
     </row>
     <row r="13" ht="12.75" customHeight="1" s="17">
-      <c r="A13" s="9" t="n"/>
-      <c r="B13" s="10" t="n"/>
-      <c r="C13" s="14" t="n"/>
-      <c r="D13" s="14" t="n"/>
-      <c r="E13" s="10" t="n"/>
-      <c r="F13" s="10" t="n"/>
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>หากต้องการคัดลอกไฟล์ Public Key ของเครื่องเราไปยังเซิร์ฟเวอร์เพื่อให้ล็อกอินด้วย Key สำเร็จโดยอัตโนมัติ ควรใช้คำสั่งใด?</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>ssh-copy-id</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>ssh-add-key</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>scp-key</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>ssh-install</t>
+        </is>
+      </c>
       <c r="G13" s="14" t="n"/>
-      <c r="H13" s="11" t="n"/>
-      <c r="I13" s="10" t="n"/>
+      <c r="H13" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="10" t="n">
+        <v>20</v>
+      </c>
       <c r="J13" s="10" t="n"/>
     </row>
     <row r="14" ht="12.75" customHeight="1" s="17">
-      <c r="A14" s="9" t="n"/>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="14" t="n"/>
-      <c r="D14" s="14" t="n"/>
-      <c r="E14" s="10" t="n"/>
-      <c r="F14" s="10" t="n"/>
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>สิทธิ์ตัวเลขฐานแปด (Octal Mode) ของไฟล์ข้อความ '-rwx------' คือเลขใด?</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>700</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>755</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>644</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>600</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="n"/>
-      <c r="H14" s="11" t="n"/>
-      <c r="I14" s="10" t="n"/>
+      <c r="H14" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" s="10" t="n">
+        <v>20</v>
+      </c>
       <c r="J14" s="10" t="n"/>
     </row>
     <row r="15" ht="12.75" customHeight="1" s="17">
-      <c r="A15" s="9" t="n"/>
-      <c r="B15" s="10" t="n"/>
-      <c r="C15" s="14" t="n"/>
-      <c r="D15" s="14" t="n"/>
-      <c r="E15" s="10" t="n"/>
-      <c r="F15" s="10" t="n"/>
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>หากหน้าเว็บไฟล์ index.html ในโฟลเดอร์ /var/www/html/ ถูกกำหนดสิทธิ์เป็น '600' (rw-------) และเป็นของ root ผู้ใช้งานทั่วไปที่เปิดเว็บเบราว์เซอร์จะพบข้อผิดพลาดใด?</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="inlineStr">
+        <is>
+          <t>403 Forbidden (เนื่องจากผู้ใช้งาน Nginx/Others อ่านไฟล์ไม่ได้)</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="inlineStr">
+        <is>
+          <t>404 Not Found (เนื่องจากไฟล์ถูกลบ)</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>500 Internal Server Error (เนื่องจากสคริปต์พัง)</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>200 OK (แสดงผลปกติ)</t>
+        </is>
+      </c>
       <c r="G15" s="14" t="n"/>
-      <c r="H15" s="11" t="n"/>
-      <c r="I15" s="10" t="n"/>
+      <c r="H15" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="J15" s="10" t="n"/>
     </row>
     <row r="16" ht="12.75" customHeight="1" s="17">
-      <c r="A16" s="9" t="n"/>
-      <c r="B16" s="10" t="n"/>
-      <c r="C16" s="14" t="n"/>
-      <c r="D16" s="14" t="n"/>
-      <c r="E16" s="10" t="n"/>
-      <c r="F16" s="10" t="n"/>
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>สิทธิ์แบบใดที่เรียกว่า 'Dangerous Permissions' (สิทธิ์อันตรายที่สุด) ที่ไม่ควรนำมาใช้บน Production Server โดยเด็ดขาด?</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="inlineStr">
+        <is>
+          <t>777 (rwxrwxrwx)</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="inlineStr">
+        <is>
+          <t>755 (rwxr-xr-x)</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>644 (rw-r--r--)</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>600 (rw-------)</t>
+        </is>
+      </c>
       <c r="G16" s="14" t="n"/>
-      <c r="H16" s="11" t="n"/>
-      <c r="I16" s="10" t="n"/>
+      <c r="H16" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="10" t="n">
+        <v>20</v>
+      </c>
       <c r="J16" s="10" t="n"/>
     </row>
     <row r="17" ht="12.75" customHeight="1" s="17">
-      <c r="A17" s="9" t="n"/>
-      <c r="B17" s="10" t="n"/>
-      <c r="C17" s="14" t="n"/>
-      <c r="D17" s="14" t="n"/>
-      <c r="E17" s="10" t="n"/>
-      <c r="F17" s="10" t="n"/>
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>คำสั่งใดใช้สลับบัญชีผู้ใช้งานจาก root ไปเป็นบัญชี 'student01' โดยดึงค่าสภาพแวดล้อมระบบ (Environment Variables) ของ student01 มาด้วย?</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>su - student01</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>su student01</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>switch student01</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>login student01</t>
+        </is>
+      </c>
       <c r="G17" s="14" t="n"/>
-      <c r="H17" s="11" t="n"/>
-      <c r="I17" s="10" t="n"/>
+      <c r="H17" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="10" t="n">
+        <v>25</v>
+      </c>
       <c r="J17" s="10" t="n"/>
     </row>
     <row r="18" ht="12.75" customHeight="1" s="17">
-      <c r="A18" s="9" t="n"/>
-      <c r="B18" s="10" t="n"/>
-      <c r="C18" s="14" t="n"/>
-      <c r="D18" s="14" t="n"/>
-      <c r="E18" s="10" t="n"/>
-      <c r="F18" s="10" t="n"/>
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>คำสั่งตรวจสอบความถูกต้องของไวยากรณ์ (Syntax Test) ในไฟล์ตั้งค่า SSH Server ก่อนสั่ง reload บริการคือคำสั่งใด?</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>sudo sshd -t</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
+        <is>
+          <t>sudo systemctl check ssh</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>sudo ssh -test</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>sudo service sshd verify</t>
+        </is>
+      </c>
       <c r="G18" s="14" t="n"/>
-      <c r="H18" s="11" t="n"/>
-      <c r="I18" s="10" t="n"/>
+      <c r="H18" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="10" t="n">
+        <v>25</v>
+      </c>
       <c r="J18" s="10" t="n"/>
     </row>
     <row r="19" ht="12.75" customHeight="1" s="17">
-      <c r="A19" s="9" t="n"/>
-      <c r="B19" s="10" t="n"/>
-      <c r="C19" s="14" t="n"/>
-      <c r="D19" s="14" t="n"/>
-      <c r="E19" s="10" t="n"/>
-      <c r="F19" s="10" t="n"/>
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>หากต้องการโหลดไฟล์ตั้งค่าของ SSH Server ใหม่ (Reload) เพื่อให้การตั้งค่ามีผลโดยไม่มีการตัดการเชื่อมต่อของผู้ใช้ปัจจุบัน ควรใช้คำสั่งใด?</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>sudo systemctl reload ssh</t>
+        </is>
+      </c>
+      <c r="D19" s="14" t="inlineStr">
+        <is>
+          <t>sudo systemctl restart ssh</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>sudo systemctl stop ssh</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>sudo systemctl enable ssh</t>
+        </is>
+      </c>
       <c r="G19" s="14" t="n"/>
-      <c r="H19" s="11" t="n"/>
-      <c r="I19" s="10" t="n"/>
+      <c r="H19" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="10" t="n">
+        <v>25</v>
+      </c>
       <c r="J19" s="10" t="n"/>
     </row>
     <row r="20" ht="12.75" customHeight="1" s="17">
-      <c r="A20" s="9" t="n"/>
-      <c r="B20" s="10" t="n"/>
-      <c r="C20" s="14" t="n"/>
-      <c r="D20" s="14" t="n"/>
-      <c r="E20" s="10" t="n"/>
-      <c r="F20" s="10" t="n"/>
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>ในสิทธิ์ระบบลินุกซ์ สัญลักษณ์ 'o' (Others) หมายถึงกลุ่มเป้าหมายในข้อใด?</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="inlineStr">
+        <is>
+          <t>ผู้ใช้ทุกคนที่เหลืออยู่ในระบบนอกเหนือจาก Owner และ Group</t>
+        </is>
+      </c>
+      <c r="D20" s="14" t="inlineStr">
+        <is>
+          <t>เจ้าของไฟล์ (Owner)</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>สมาชิกในกลุ่ม (Group)</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>สิทธิ์พิเศษระบบ (root)</t>
+        </is>
+      </c>
       <c r="G20" s="14" t="n"/>
-      <c r="H20" s="11" t="n"/>
-      <c r="I20" s="10" t="n"/>
+      <c r="H20" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="10" t="n">
+        <v>20</v>
+      </c>
       <c r="J20" s="10" t="n"/>
     </row>
     <row r="21" ht="12.75" customHeight="1" s="17">
-      <c r="A21" s="9" t="n"/>
-      <c r="B21" s="10" t="n"/>
-      <c r="C21" s="14" t="n"/>
-      <c r="D21" s="14" t="n"/>
-      <c r="E21" s="10" t="n"/>
-      <c r="F21" s="10" t="n"/>
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>หากต้องการเปลี่ยนกลุ่มเจ้าของไฟล์ (Group Ownership) เพียงอย่างเดียวของไฟล์ report.txt โดยไม่เปลี่ยนเจ้าของไฟล์ตัวจริง ควรใช้คำสั่งใด?</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>sudo chgrp www-data report.txt</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="inlineStr">
+        <is>
+          <t>sudo chown www-data report.txt</t>
+        </is>
+      </c>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>sudo chmod g+w report.txt</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>sudo usermod -aG www-data report.txt</t>
+        </is>
+      </c>
       <c r="G21" s="14" t="n"/>
-      <c r="H21" s="11" t="n"/>
-      <c r="I21" s="10" t="n"/>
+      <c r="H21" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="10" t="n">
+        <v>25</v>
+      </c>
       <c r="J21" s="10" t="n"/>
     </row>
     <row r="22" ht="12.75" customHeight="1" s="17">
-      <c r="A22" s="9" t="n"/>
-      <c r="B22" s="10" t="n"/>
-      <c r="C22" s="14" t="n"/>
-      <c r="D22" s="14" t="n"/>
-      <c r="E22" s="10" t="n"/>
-      <c r="F22" s="10" t="n"/>
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>ไฟล์ที่ใช้เก็บรายชื่อ Public Keys ของคอมพิวเตอร์ภายนอกที่ได้รับอนุญาตให้ล็อกอินเข้าเซิร์ฟเวอร์ของแต่ละผู้ใช้ในระบบ จะถูกบันทึกไว้ในพาธใดบนเซิร์ฟเวอร์?</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Multiple Choice</t>
+        </is>
+      </c>
+      <c r="C22" s="14" t="inlineStr">
+        <is>
+          <t>~/.ssh/authorized_keys</t>
+        </is>
+      </c>
+      <c r="D22" s="14" t="inlineStr">
+        <is>
+          <t>~/.ssh/id_ed25519.pub</t>
+        </is>
+      </c>
+      <c r="E22" s="10" t="inlineStr">
+        <is>
+          <t>/etc/ssh/ssh_host_key</t>
+        </is>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>/var/log/auth.log</t>
+        </is>
+      </c>
       <c r="G22" s="14" t="n"/>
-      <c r="H22" s="11" t="n"/>
-      <c r="I22" s="10" t="n"/>
+      <c r="H22" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="J22" s="10" t="n"/>
     </row>
     <row r="23" ht="12.75" customHeight="1" s="17">

</xml_diff>